<commit_message>
Record keiba and kyotei sample through-test writes on September sheets
Co-authored-by: tama357 <tama357@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/個人予想/excel/競艇_予想記入シート_2026年9月.xlsx
+++ b/個人予想/excel/競艇_予想記入シート_2026年9月.xlsx
@@ -947,25 +947,25 @@
       </c>
       <c r="E3" s="41" t="inlineStr">
         <is>
-          <t>多摩川</t>
+          <t>児島</t>
         </is>
       </c>
       <c r="F3" s="77" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G3" s="78" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="H3" s="42" t="inlineStr">
         <is>
-          <t>1-2-456</t>
+          <t>1-3-245</t>
         </is>
       </c>
       <c r="I3" s="42" t="inlineStr">
         <is>
-          <t>1-3-456 1-4-56</t>
+          <t>1-6-245 1-2-45</t>
         </is>
       </c>
       <c r="J3" s="79" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="K3" s="42" t="inlineStr">
         <is>
-          <t>[予想しやすさ90] 軸1番。1号艇が能力・モーターとも上位。イン逃げ想定。 / 想定:1号艇逃げ、2・3着は2-3-4 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ93] 軸1番。1号艇軸（中村日向）、全国勝率7.17、モーター2連対39.8、展示6.8、最人気オッズ6.1 / 想定:1号艇が主導。2着候補3・6 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L3" s="43" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="C4" s="35" t="inlineStr">
         <is>
-          <t>中穴</t>
+          <t>鉄板</t>
         </is>
       </c>
       <c r="D4" s="35" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E4" s="35" t="inlineStr">
@@ -1011,21 +1011,21 @@
         </is>
       </c>
       <c r="F4" s="82" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G4" s="83" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:58</t>
         </is>
       </c>
       <c r="H4" s="36" t="inlineStr">
         <is>
-          <t>2-1-456</t>
+          <t>1-3-246</t>
         </is>
       </c>
       <c r="I4" s="36" t="inlineStr">
         <is>
-          <t>2-3-456 2-4-56</t>
+          <t>1-5-246 1-2-46</t>
         </is>
       </c>
       <c r="J4" s="84" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="K4" s="36" t="inlineStr">
         <is>
-          <t>[予想しやすさ82] 軸2番 / 想定:軸2先行〜差し切り想定 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ91] 軸1番。1号艇軸（小林一樹）、全国勝率5.76、モーター2連対70.0、展示6.66、最人気オッズ3.2 / 想定:1号艇が主導。2着候補3・5 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L4" s="38" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>中穴</t>
+          <t>鉄板</t>
         </is>
       </c>
       <c r="D5" s="35" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -1071,21 +1071,21 @@
         </is>
       </c>
       <c r="F5" s="82" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G5" s="83" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="H5" s="36" t="inlineStr">
         <is>
-          <t>1-2-356</t>
+          <t>1-4-256</t>
         </is>
       </c>
       <c r="I5" s="36" t="inlineStr">
         <is>
-          <t>1-4-356 1-3-56</t>
+          <t>1-3-256 1-2-56</t>
         </is>
       </c>
       <c r="J5" s="84" t="n">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="K5" s="36" t="inlineStr">
         <is>
-          <t>[予想しやすさ78] 軸1番 / 想定:軸1先行〜差し切り想定 / リスク:evenly_matched</t>
+          <t>[予想しやすさ90] 軸1番。1号艇軸（三浦永理）、全国勝率7.31、モーター2連対40.57、展示6.65、最人気オッズ6.7 / 想定:1号艇が主導。2着候補4・3 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L5" s="38" t="inlineStr">
@@ -1117,35 +1117,35 @@
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>中穴</t>
+          <t>鉄板</t>
         </is>
       </c>
       <c r="D6" s="35" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E6" s="35" t="inlineStr">
         <is>
-          <t>住之江</t>
+          <t>蒲郡</t>
         </is>
       </c>
       <c r="F6" s="82" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G6" s="83" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="H6" s="36" t="inlineStr">
         <is>
-          <t>1-2-456</t>
+          <t>1-4-256</t>
         </is>
       </c>
       <c r="I6" s="36" t="inlineStr">
         <is>
-          <t>1-3-456 1-4-56</t>
+          <t>1-3-256 1-2-56</t>
         </is>
       </c>
       <c r="J6" s="84" t="n">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="K6" s="36" t="inlineStr">
         <is>
-          <t>[予想しやすさ76] 軸1番 / 想定:軸1先行〜差し切り想定 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ88] 軸1番。1号艇軸（山田晃大）、全国勝率5.82、モーター2連対50.0、展示6.67、最人気オッズ5.6 / 想定:1号艇が主導。2着候補4・3 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L6" s="38" t="inlineStr">
@@ -1177,35 +1177,35 @@
       </c>
       <c r="C7" s="49" t="inlineStr">
         <is>
-          <t>中穴</t>
+          <t>鉄板</t>
         </is>
       </c>
       <c r="D7" s="49" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>常滑</t>
+          <t>児島</t>
         </is>
       </c>
       <c r="F7" s="87" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G7" s="88" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="H7" s="50" t="inlineStr">
         <is>
-          <t>1-2-456</t>
+          <t>1-6-234</t>
         </is>
       </c>
       <c r="I7" s="50" t="inlineStr">
         <is>
-          <t>1-3-456 1-4-56</t>
+          <t>1-5-234 1-2-34</t>
         </is>
       </c>
       <c r="J7" s="89" t="n">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="K7" s="50" t="inlineStr">
         <is>
-          <t>[予想しやすさ75] 軸1番 / 想定:軸1先行〜差し切り想定 / リスク:data_shortage</t>
+          <t>[予想しやすさ87] 軸1番。1号艇軸（石倉洋行）、全国勝率7.17、モーター2連対35.42、展示6.85、最人気オッズ7.6 / 想定:1号艇が主導。2着候補6・5 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L7" s="51" t="inlineStr">

</xml_diff>

<commit_message>
Split personal predictions into JRA, NAR, and kyotei
Use six Excel workbooks with separate state and learning data.
Submission keirin under 競輪予想/ is unchanged. Drive is not updated.

Co-authored-by: tama357 <tama357@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/個人予想/excel/競艇_予想記入シート_2026年9月.xlsx
+++ b/個人予想/excel/競艇_予想記入シート_2026年9月.xlsx
@@ -947,25 +947,25 @@
       </c>
       <c r="E3" s="41" t="inlineStr">
         <is>
-          <t>児島</t>
+          <t>多摩川</t>
         </is>
       </c>
       <c r="F3" s="77" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G3" s="78" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="H3" s="42" t="inlineStr">
         <is>
-          <t>1-3-245</t>
+          <t>1-2-456</t>
         </is>
       </c>
       <c r="I3" s="42" t="inlineStr">
         <is>
-          <t>1-6-245 1-2-45</t>
+          <t>1-3-456 1-4-56</t>
         </is>
       </c>
       <c r="J3" s="79" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="K3" s="42" t="inlineStr">
         <is>
-          <t>[予想しやすさ93] 軸1番。1号艇軸（中村日向）、全国勝率7.17、モーター2連対39.8、展示6.8、最人気オッズ6.1 / 想定:1号艇が主導。2着候補3・6 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ90] 軸1番。1号艇が能力・モーターとも上位。イン逃げ想定。 / 想定:1号艇逃げ、2・3着は2-3-4 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L3" s="43" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="C4" s="35" t="inlineStr">
         <is>
-          <t>鉄板</t>
+          <t>中穴</t>
         </is>
       </c>
       <c r="D4" s="35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E4" s="35" t="inlineStr">
@@ -1011,21 +1011,21 @@
         </is>
       </c>
       <c r="F4" s="82" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G4" s="83" t="inlineStr">
         <is>
-          <t>17:58</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="H4" s="36" t="inlineStr">
         <is>
-          <t>1-3-246</t>
+          <t>2-1-456</t>
         </is>
       </c>
       <c r="I4" s="36" t="inlineStr">
         <is>
-          <t>1-5-246 1-2-46</t>
+          <t>2-3-456 2-4-56</t>
         </is>
       </c>
       <c r="J4" s="84" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="K4" s="36" t="inlineStr">
         <is>
-          <t>[予想しやすさ91] 軸1番。1号艇軸（小林一樹）、全国勝率5.76、モーター2連対70.0、展示6.66、最人気オッズ3.2 / 想定:1号艇が主導。2着候補3・5 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ82] 軸2番 / 想定:軸2先行〜差し切り想定 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L4" s="38" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>鉄板</t>
+          <t>中穴</t>
         </is>
       </c>
       <c r="D5" s="35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -1071,21 +1071,21 @@
         </is>
       </c>
       <c r="F5" s="82" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G5" s="83" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="H5" s="36" t="inlineStr">
         <is>
-          <t>1-4-256</t>
+          <t>1-2-356</t>
         </is>
       </c>
       <c r="I5" s="36" t="inlineStr">
         <is>
-          <t>1-3-256 1-2-56</t>
+          <t>1-4-356 1-3-56</t>
         </is>
       </c>
       <c r="J5" s="84" t="n">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="K5" s="36" t="inlineStr">
         <is>
-          <t>[予想しやすさ90] 軸1番。1号艇軸（三浦永理）、全国勝率7.31、モーター2連対40.57、展示6.65、最人気オッズ6.7 / 想定:1号艇が主導。2着候補4・3 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ78] 軸1番 / 想定:軸1先行〜差し切り想定 / リスク:evenly_matched</t>
         </is>
       </c>
       <c r="L5" s="38" t="inlineStr">
@@ -1117,35 +1117,35 @@
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>鉄板</t>
+          <t>中穴</t>
         </is>
       </c>
       <c r="D6" s="35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E6" s="35" t="inlineStr">
         <is>
-          <t>蒲郡</t>
+          <t>住之江</t>
         </is>
       </c>
       <c r="F6" s="82" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G6" s="83" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="H6" s="36" t="inlineStr">
         <is>
-          <t>1-4-256</t>
+          <t>1-2-456</t>
         </is>
       </c>
       <c r="I6" s="36" t="inlineStr">
         <is>
-          <t>1-3-256 1-2-56</t>
+          <t>1-3-456 1-4-56</t>
         </is>
       </c>
       <c r="J6" s="84" t="n">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="K6" s="36" t="inlineStr">
         <is>
-          <t>[予想しやすさ88] 軸1番。1号艇軸（山田晃大）、全国勝率5.82、モーター2連対50.0、展示6.67、最人気オッズ5.6 / 想定:1号艇が主導。2着候補4・3 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ76] 軸1番 / 想定:軸1先行〜差し切り想定 / リスク:展開変化に注意</t>
         </is>
       </c>
       <c r="L6" s="38" t="inlineStr">
@@ -1177,35 +1177,35 @@
       </c>
       <c r="C7" s="49" t="inlineStr">
         <is>
-          <t>鉄板</t>
+          <t>中穴</t>
         </is>
       </c>
       <c r="D7" s="49" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>児島</t>
+          <t>常滑</t>
         </is>
       </c>
       <c r="F7" s="87" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G7" s="88" t="inlineStr">
         <is>
-          <t>14:23</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="H7" s="50" t="inlineStr">
         <is>
-          <t>1-6-234</t>
+          <t>1-2-456</t>
         </is>
       </c>
       <c r="I7" s="50" t="inlineStr">
         <is>
-          <t>1-5-234 1-2-34</t>
+          <t>1-3-456 1-4-56</t>
         </is>
       </c>
       <c r="J7" s="89" t="n">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="K7" s="50" t="inlineStr">
         <is>
-          <t>[予想しやすさ87] 軸1番。1号艇軸（石倉洋行）、全国勝率7.17、モーター2連対35.42、展示6.85、最人気オッズ7.6 / 想定:1号艇が主導。2着候補6・5 / リスク:展開変化に注意</t>
+          <t>[予想しやすさ75] 軸1番 / 想定:軸1先行〜差し切り想定 / リスク:data_shortage</t>
         </is>
       </c>
       <c r="L7" s="51" t="inlineStr">

</xml_diff>